<commit_message>
Update RM fallback to use sheet Sender_Name when Sender_ID mapping is unavailable
</commit_message>
<xml_diff>
--- a/RM_standard_name.xlsx
+++ b/RM_standard_name.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chipmonggroup-my.sharepoint.com/personal/tra_troeurn_chipmongbank_com/Documents/Documents/Streamlit_customer_data/STEAMLIB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36F2271D-729C-448F-B6D8-6BD94BDB86AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{36F2271D-729C-448F-B6D8-6BD94BDB86AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B8613E8-3EE8-4306-B4A8-C2E7C5A8C1A6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4B6BB340-08E3-4F70-A32A-D433B1207051}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="287">
   <si>
     <t>Heang Kimhour</t>
   </si>
@@ -883,6 +883,21 @@
   </si>
   <si>
     <t>Sender_ID</t>
+  </si>
+  <si>
+    <t>KHON Vichet</t>
+  </si>
+  <si>
+    <t>KROURCH Samnang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DY Rithy </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIN Pov </t>
+  </si>
+  <si>
+    <t>SUM Channy</t>
   </si>
 </sst>
 </file>
@@ -974,7 +989,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -982,11 +997,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1001,11 +1044,42 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1030,30 +1104,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1068,10 +1118,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF37F533-85FF-4050-985D-CFC1A8D7C072}" name="Table1" displayName="Table1" ref="A1:B314" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:B314" xr:uid="{DF37F533-85FF-4050-985D-CFC1A8D7C072}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF37F533-85FF-4050-985D-CFC1A8D7C072}" name="Table1" displayName="Table1" ref="A1:B319" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:B319" xr:uid="{DF37F533-85FF-4050-985D-CFC1A8D7C072}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{37F919A4-1A99-492F-A9CA-815089180E40}" name="Sender_ID" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{37F919A4-1A99-492F-A9CA-815089180E40}" name="Sender_ID" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{3304CF29-C268-49E1-A4D7-23ABC55BC106}" name="Standard_Name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1375,7 +1425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52D3B542-963A-437D-B610-55E06D5D28F8}">
-  <dimension ref="A1:B314"/>
+  <dimension ref="A1:B319"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -3892,6 +3942,44 @@
         <v>279</v>
       </c>
     </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="13">
+        <v>1409843986</v>
+      </c>
+      <c r="B315" s="14" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="13">
+        <v>8377847944</v>
+      </c>
+      <c r="B316" s="14" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2">
+        <v>1362093252</v>
+      </c>
+      <c r="B317" s="12" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="2">
+        <v>1052771544</v>
+      </c>
+      <c r="B318" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2">
+      <c r="A319" s="13"/>
+      <c r="B319" s="14" t="s">
+        <v>286</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>